<commit_message>
Update HemaCDS 2.0 Multiple Myeloma Electrophoresis UI
</commit_message>
<xml_diff>
--- a/HemaCDS_2.0_Multiple Myeloma_Chemotherapy/HemaCDS2.0_Mutiple Myeloma.xlsx
+++ b/HemaCDS_2.0_Multiple Myeloma_Chemotherapy/HemaCDS2.0_Mutiple Myeloma.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\내 드라이브\Antigravity\HemaCDS_2.0_Multiple Myeloma_Chemotherapy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B4FAEB4-D6DC-44EA-8345-994589D8AD11}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B525BEF3-FAAC-4D8B-8723-801BC174E69B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25365" windowHeight="8565" xr2:uid="{4603E7B1-FC8D-44F2-B512-2B7619F217F2}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="151">
   <si>
     <t>Daratumumab</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -413,10 +413,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>D-VTD (Bortezomib weekly)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>QW2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -430,10 +426,6 @@
   </si>
   <si>
     <t>BiQW2, QW4, QW3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>C2QW3, QW3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -557,8 +549,60 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>CELMoD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mezigmoide</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>C21</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1 mg, 0.6 mg, 0.3 mg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mezigdomide</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Carfilzomib</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1.0 mg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>C1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>56 mg/m2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>20 mg/m2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>QW2F8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D8, 15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <r>
-      <t>D-VTD</t>
+      <t>C1, C2, QW3, Q2W, C2QW3, QW3</t>
     </r>
     <r>
       <rPr>
@@ -568,20 +612,52 @@
         <family val="2"/>
         <charset val="129"/>
       </rPr>
-      <t xml:space="preserve"> (Bortezomib biweekly)</t>
+      <t>, QW2F8</t>
     </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>CELMoD</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Mezigmoide</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M</t>
+    <t>QWF8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2-12</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>13-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Q2W</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mezi-Kd</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D-VTd (Bortezomib weekly)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D-VTd (Bortezomib biweekly)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ezi</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -589,7 +665,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -634,6 +710,13 @@
       <family val="2"/>
       <charset val="129"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Noto Sans Korean Regular"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -657,7 +740,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -679,19 +762,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1049,7 +1138,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1066,7 +1155,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1083,7 +1172,7 @@
         <v>26</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1100,7 +1189,7 @@
         <v>7</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1117,7 +1206,7 @@
         <v>11</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1168,7 +1257,7 @@
         <v>20</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1185,54 +1274,58 @@
         <v>23</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="4"/>
+      <c r="E11" s="4" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>117</v>
-      </c>
       <c r="D13" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1249,7 +1342,7 @@
         <v>29</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1257,16 +1350,16 @@
         <v>43</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="E15" s="4" t="s">
         <v>121</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1283,7 +1376,7 @@
         <v>32</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1300,7 +1393,7 @@
         <v>35</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:6" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1317,7 +1410,7 @@
         <v>38</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:6" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1334,7 +1427,7 @@
         <v>47</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1446,7 +1539,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BCB5F65-E379-4517-9A0D-89CF0C09D06D}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.625" customWidth="1"/>
@@ -1482,7 +1575,7 @@
         <v>94</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -1526,96 +1619,104 @@
       </c>
     </row>
     <row r="10" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>75</v>
+      <c r="A10" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>111</v>
+        <v>106</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:B1" xr:uid="{D4A9A49E-0364-4B1A-BA6B-37CA9B42F8A6}">
-    <sortState ref="A2:B19">
+    <sortState ref="A2:B20">
       <sortCondition ref="A1"/>
     </sortState>
   </autoFilter>
@@ -1626,7 +1727,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{710D1B9E-2C33-411D-90E0-19C442F97FD6}">
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.625" style="6" customWidth="1"/>
@@ -1635,468 +1736,611 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+    </row>
+    <row r="2" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="12">
+        <v>28</v>
+      </c>
+      <c r="E2" s="9"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+    </row>
+    <row r="3" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="10"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+    </row>
+    <row r="4" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="10"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+    </row>
+    <row r="5" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="10"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+    </row>
+    <row r="6" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="10"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+    </row>
+    <row r="7" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="10"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+    </row>
+    <row r="8" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="10"/>
+      <c r="B8" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="12">
+        <v>28</v>
+      </c>
+      <c r="E8" s="9"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+    </row>
+    <row r="9" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="10"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="10"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="10"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+    </row>
+    <row r="12" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="10"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+    </row>
+    <row r="13" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="10"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+    </row>
+    <row r="14" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="10"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+    </row>
+    <row r="15" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="12">
+        <v>28</v>
+      </c>
+      <c r="E15" s="9"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+    </row>
+    <row r="16" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="10"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+    </row>
+    <row r="17" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="10"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+    </row>
+    <row r="18" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="10"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E18" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+    </row>
+    <row r="19" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="10"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="K19" s="2"/>
+    </row>
+    <row r="20" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="10"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="10"/>
+      <c r="B21" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" s="12">
+        <v>28</v>
+      </c>
+      <c r="E21" s="9"/>
+    </row>
+    <row r="22" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="10"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="10"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="E23" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="C2" s="8" t="s">
+    </row>
+    <row r="24" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="10"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="10"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="10"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="10"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="C28" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="8">
+      <c r="D28" s="12">
         <v>28</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="9"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="8" t="s">
+      <c r="E28" s="9"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A29" s="10"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D29" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E29" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="9"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="E4" s="3" t="s">
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A30" s="10"/>
+      <c r="B30" s="11"/>
+      <c r="C30" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="E30" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="K4" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" s="3" t="s">
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A31" s="10"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A32" s="10"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="10"/>
+      <c r="B33" s="11"/>
+      <c r="C33" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D33" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E33" s="9" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="10"/>
+      <c r="B34" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D34" s="12">
+        <v>28</v>
+      </c>
+      <c r="E34" s="9"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="10"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="10"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="E36" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="K5" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="9"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="5" t="s">
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="10"/>
+      <c r="B37" s="11"/>
+      <c r="C37" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="10"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="9"/>
-      <c r="B8" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="8" t="s">
+      <c r="D38" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="10"/>
+      <c r="B39" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="C39" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D39" s="12">
         <v>28</v>
       </c>
-      <c r="K8" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="8" t="s">
+      <c r="E39" s="9"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="10"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D40" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E40" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="K9" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" s="3" t="s">
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="10"/>
+      <c r="B41" s="11"/>
+      <c r="C41" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="10"/>
+      <c r="B42" s="11"/>
+      <c r="C42" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="10"/>
+      <c r="B43" s="11"/>
+      <c r="C43" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D43" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="9"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="9"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="9"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D15" s="8">
-        <v>28</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="9"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="9"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="9"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="9"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="9"/>
-      <c r="B21" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D21" s="8">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="9"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="9"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="9"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="9"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="9"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="E43" s="9" t="s">
+        <v>123</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="10">
+    <mergeCell ref="B28:B33"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="B39:B43"/>
+    <mergeCell ref="A28:A43"/>
     <mergeCell ref="A2:A14"/>
     <mergeCell ref="A15:A27"/>
     <mergeCell ref="B2:B7"/>

</xml_diff>